<commit_message>
Update for Study Code
</commit_message>
<xml_diff>
--- a/Study_2_Early_Late_Correction/data/correction_raw_data.xlsx
+++ b/Study_2_Early_Late_Correction/data/correction_raw_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\59784\Desktop\StatsError\Final Results\Early_Late_Correctness\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\59784\Desktop\Stats Learning\Data_Analysis\LLM-Stats-Learning\Study_2_Early_Late_Correction\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC410F7F-076C-47CB-9B2F-23B854CCC328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12800" yWindow="790" windowWidth="12700" windowHeight="15110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2970" yWindow="4065" windowWidth="28800" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,9 +19,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -365,7 +362,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -644,9 +641,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BS179"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -861,7 +858,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>70</v>
       </c>
@@ -1042,7 +1039,7 @@
       <c r="BR2" s="5"/>
       <c r="BS2" s="5"/>
     </row>
-    <row r="3" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -1257,7 +1254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>70</v>
       </c>
@@ -1438,7 +1435,7 @@
       <c r="BR4" s="10"/>
       <c r="BS4" s="10"/>
     </row>
-    <row r="5" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -1619,7 +1616,7 @@
       <c r="BR5" s="10"/>
       <c r="BS5" s="10"/>
     </row>
-    <row r="6" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>70</v>
       </c>
@@ -1800,7 +1797,7 @@
       <c r="BR6" s="10"/>
       <c r="BS6" s="10"/>
     </row>
-    <row r="7" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>70</v>
       </c>
@@ -1981,7 +1978,7 @@
       <c r="BR7" s="10"/>
       <c r="BS7" s="10"/>
     </row>
-    <row r="8" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>72</v>
       </c>
@@ -2162,7 +2159,7 @@
       <c r="BR8" s="10"/>
       <c r="BS8" s="10"/>
     </row>
-    <row r="9" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>72</v>
       </c>
@@ -2343,7 +2340,7 @@
       <c r="BR9" s="10"/>
       <c r="BS9" s="10"/>
     </row>
-    <row r="10" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>70</v>
       </c>
@@ -2558,7 +2555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>70</v>
       </c>
@@ -2773,7 +2770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>71</v>
       </c>
@@ -2954,7 +2951,7 @@
       <c r="BR12" s="10"/>
       <c r="BS12" s="10"/>
     </row>
-    <row r="13" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>70</v>
       </c>
@@ -3135,7 +3132,7 @@
       <c r="BR13" s="10"/>
       <c r="BS13" s="10"/>
     </row>
-    <row r="14" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>72</v>
       </c>
@@ -3316,7 +3313,7 @@
       <c r="BR14" s="10"/>
       <c r="BS14" s="10"/>
     </row>
-    <row r="15" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>70</v>
       </c>
@@ -3531,7 +3528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>72</v>
       </c>
@@ -3712,7 +3709,7 @@
       <c r="BR16" s="10"/>
       <c r="BS16" s="10"/>
     </row>
-    <row r="17" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>72</v>
       </c>
@@ -3893,7 +3890,7 @@
       <c r="BR17" s="10"/>
       <c r="BS17" s="10"/>
     </row>
-    <row r="18" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>70</v>
       </c>
@@ -4074,7 +4071,7 @@
       <c r="BR18" s="10"/>
       <c r="BS18" s="10"/>
     </row>
-    <row r="19" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -4289,7 +4286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -4470,7 +4467,7 @@
       <c r="BR20" s="10"/>
       <c r="BS20" s="10"/>
     </row>
-    <row r="21" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -4651,7 +4648,7 @@
       <c r="BR21" s="10"/>
       <c r="BS21" s="10"/>
     </row>
-    <row r="22" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>70</v>
       </c>
@@ -4832,7 +4829,7 @@
       <c r="BR22" s="10"/>
       <c r="BS22" s="10"/>
     </row>
-    <row r="23" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>71</v>
       </c>
@@ -5013,7 +5010,7 @@
       <c r="BR23" s="10"/>
       <c r="BS23" s="10"/>
     </row>
-    <row r="24" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>70</v>
       </c>
@@ -5194,7 +5191,7 @@
       <c r="BR24" s="10"/>
       <c r="BS24" s="10"/>
     </row>
-    <row r="25" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>72</v>
       </c>
@@ -5375,7 +5372,7 @@
       <c r="BR25" s="10"/>
       <c r="BS25" s="10"/>
     </row>
-    <row r="26" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>70</v>
       </c>
@@ -5556,7 +5553,7 @@
       <c r="BR26" s="10"/>
       <c r="BS26" s="10"/>
     </row>
-    <row r="27" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>72</v>
       </c>
@@ -5737,7 +5734,7 @@
       <c r="BR27" s="10"/>
       <c r="BS27" s="10"/>
     </row>
-    <row r="28" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>72</v>
       </c>
@@ -5952,7 +5949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>72</v>
       </c>
@@ -6167,7 +6164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>71</v>
       </c>
@@ -6348,7 +6345,7 @@
       <c r="BR30" s="10"/>
       <c r="BS30" s="10"/>
     </row>
-    <row r="31" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>71</v>
       </c>
@@ -6529,7 +6526,7 @@
       <c r="BR31" s="10"/>
       <c r="BS31" s="10"/>
     </row>
-    <row r="32" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>71</v>
       </c>
@@ -6710,7 +6707,7 @@
       <c r="BR32" s="10"/>
       <c r="BS32" s="10"/>
     </row>
-    <row r="33" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>70</v>
       </c>
@@ -6891,7 +6888,7 @@
       <c r="BR33" s="10"/>
       <c r="BS33" s="10"/>
     </row>
-    <row r="34" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>71</v>
       </c>
@@ -7106,7 +7103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>72</v>
       </c>
@@ -7287,7 +7284,7 @@
       <c r="BR35" s="10"/>
       <c r="BS35" s="10"/>
     </row>
-    <row r="36" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>71</v>
       </c>
@@ -7502,7 +7499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>71</v>
       </c>
@@ -7683,7 +7680,7 @@
       <c r="BR37" s="10"/>
       <c r="BS37" s="10"/>
     </row>
-    <row r="38" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>72</v>
       </c>
@@ -7864,7 +7861,7 @@
       <c r="BR38" s="10"/>
       <c r="BS38" s="10"/>
     </row>
-    <row r="39" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>70</v>
       </c>
@@ -8045,7 +8042,7 @@
       <c r="BR39" s="10"/>
       <c r="BS39" s="10"/>
     </row>
-    <row r="40" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>72</v>
       </c>
@@ -8226,7 +8223,7 @@
       <c r="BR40" s="10"/>
       <c r="BS40" s="10"/>
     </row>
-    <row r="41" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>71</v>
       </c>
@@ -8407,7 +8404,7 @@
       <c r="BR41" s="10"/>
       <c r="BS41" s="10"/>
     </row>
-    <row r="42" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>72</v>
       </c>
@@ -8588,7 +8585,7 @@
       <c r="BR42" s="10"/>
       <c r="BS42" s="10"/>
     </row>
-    <row r="43" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>72</v>
       </c>
@@ -8769,7 +8766,7 @@
       <c r="BR43" s="10"/>
       <c r="BS43" s="10"/>
     </row>
-    <row r="44" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>71</v>
       </c>
@@ -8950,7 +8947,7 @@
       <c r="BR44" s="10"/>
       <c r="BS44" s="10"/>
     </row>
-    <row r="45" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>72</v>
       </c>
@@ -9131,7 +9128,7 @@
       <c r="BR45" s="10"/>
       <c r="BS45" s="10"/>
     </row>
-    <row r="46" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>70</v>
       </c>
@@ -9312,7 +9309,7 @@
       <c r="BR46" s="10"/>
       <c r="BS46" s="10"/>
     </row>
-    <row r="47" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>72</v>
       </c>
@@ -9527,7 +9524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>70</v>
       </c>
@@ -9708,7 +9705,7 @@
       <c r="BR48" s="10"/>
       <c r="BS48" s="10"/>
     </row>
-    <row r="49" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>72</v>
       </c>
@@ -9889,7 +9886,7 @@
       <c r="BR49" s="10"/>
       <c r="BS49" s="10"/>
     </row>
-    <row r="50" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>70</v>
       </c>
@@ -10070,7 +10067,7 @@
       <c r="BR50" s="10"/>
       <c r="BS50" s="10"/>
     </row>
-    <row r="51" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>72</v>
       </c>
@@ -10251,7 +10248,7 @@
       <c r="BR51" s="10"/>
       <c r="BS51" s="10"/>
     </row>
-    <row r="52" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>72</v>
       </c>
@@ -10432,7 +10429,7 @@
       <c r="BR52" s="10"/>
       <c r="BS52" s="10"/>
     </row>
-    <row r="53" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>72</v>
       </c>
@@ -10647,7 +10644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>70</v>
       </c>
@@ -10828,7 +10825,7 @@
       <c r="BR54" s="10"/>
       <c r="BS54" s="10"/>
     </row>
-    <row r="55" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>70</v>
       </c>
@@ -11043,7 +11040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>71</v>
       </c>
@@ -11258,7 +11255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>70</v>
       </c>
@@ -11473,7 +11470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>72</v>
       </c>
@@ -11688,7 +11685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>72</v>
       </c>
@@ -11869,7 +11866,7 @@
       <c r="BR59" s="10"/>
       <c r="BS59" s="10"/>
     </row>
-    <row r="60" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>70</v>
       </c>
@@ -12050,7 +12047,7 @@
       <c r="BR60" s="10"/>
       <c r="BS60" s="10"/>
     </row>
-    <row r="61" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>72</v>
       </c>
@@ -12231,7 +12228,7 @@
       <c r="BR61" s="10"/>
       <c r="BS61" s="10"/>
     </row>
-    <row r="62" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>70</v>
       </c>
@@ -12412,7 +12409,7 @@
       <c r="BR62" s="10"/>
       <c r="BS62" s="10"/>
     </row>
-    <row r="63" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>70</v>
       </c>
@@ -12593,7 +12590,7 @@
       <c r="BR63" s="10"/>
       <c r="BS63" s="10"/>
     </row>
-    <row r="64" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>70</v>
       </c>
@@ -12774,7 +12771,7 @@
       <c r="BR64" s="10"/>
       <c r="BS64" s="10"/>
     </row>
-    <row r="65" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>72</v>
       </c>
@@ -12955,7 +12952,7 @@
       <c r="BR65" s="10"/>
       <c r="BS65" s="10"/>
     </row>
-    <row r="66" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>71</v>
       </c>
@@ -13136,7 +13133,7 @@
       <c r="BR66" s="10"/>
       <c r="BS66" s="10"/>
     </row>
-    <row r="67" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>71</v>
       </c>
@@ -13317,7 +13314,7 @@
       <c r="BR67" s="10"/>
       <c r="BS67" s="10"/>
     </row>
-    <row r="68" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>71</v>
       </c>
@@ -13532,7 +13529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>72</v>
       </c>
@@ -13713,7 +13710,7 @@
       <c r="BR69" s="10"/>
       <c r="BS69" s="10"/>
     </row>
-    <row r="70" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>70</v>
       </c>
@@ -13894,7 +13891,7 @@
       <c r="BR70" s="10"/>
       <c r="BS70" s="10"/>
     </row>
-    <row r="71" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>70</v>
       </c>
@@ -14075,7 +14072,7 @@
       <c r="BR71" s="10"/>
       <c r="BS71" s="10"/>
     </row>
-    <row r="72" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>72</v>
       </c>
@@ -14256,7 +14253,7 @@
       <c r="BR72" s="10"/>
       <c r="BS72" s="10"/>
     </row>
-    <row r="73" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>72</v>
       </c>
@@ -14437,7 +14434,7 @@
       <c r="BR73" s="10"/>
       <c r="BS73" s="10"/>
     </row>
-    <row r="74" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>72</v>
       </c>
@@ -14618,7 +14615,7 @@
       <c r="BR74" s="10"/>
       <c r="BS74" s="10"/>
     </row>
-    <row r="75" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>72</v>
       </c>
@@ -14799,7 +14796,7 @@
       <c r="BR75" s="10"/>
       <c r="BS75" s="10"/>
     </row>
-    <row r="76" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>70</v>
       </c>
@@ -14980,7 +14977,7 @@
       <c r="BR76" s="10"/>
       <c r="BS76" s="10"/>
     </row>
-    <row r="77" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>71</v>
       </c>
@@ -15161,7 +15158,7 @@
       <c r="BR77" s="10"/>
       <c r="BS77" s="10"/>
     </row>
-    <row r="78" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>70</v>
       </c>
@@ -15342,7 +15339,7 @@
       <c r="BR78" s="10"/>
       <c r="BS78" s="10"/>
     </row>
-    <row r="79" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>71</v>
       </c>
@@ -15557,7 +15554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>72</v>
       </c>
@@ -15772,7 +15769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>72</v>
       </c>
@@ -15953,7 +15950,7 @@
       <c r="BR81" s="10"/>
       <c r="BS81" s="10"/>
     </row>
-    <row r="82" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>71</v>
       </c>
@@ -16134,7 +16131,7 @@
       <c r="BR82" s="10"/>
       <c r="BS82" s="10"/>
     </row>
-    <row r="83" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>72</v>
       </c>
@@ -16349,7 +16346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>71</v>
       </c>
@@ -16530,7 +16527,7 @@
       <c r="BR84" s="10"/>
       <c r="BS84" s="10"/>
     </row>
-    <row r="85" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>71</v>
       </c>
@@ -16745,7 +16742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>71</v>
       </c>
@@ -16926,7 +16923,7 @@
       <c r="BR86" s="10"/>
       <c r="BS86" s="10"/>
     </row>
-    <row r="87" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>72</v>
       </c>
@@ -17141,7 +17138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>70</v>
       </c>
@@ -17356,7 +17353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>71</v>
       </c>
@@ -17537,7 +17534,7 @@
       <c r="BR89" s="10"/>
       <c r="BS89" s="10"/>
     </row>
-    <row r="90" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>72</v>
       </c>
@@ -17718,7 +17715,7 @@
       <c r="BR90" s="10"/>
       <c r="BS90" s="10"/>
     </row>
-    <row r="91" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>71</v>
       </c>
@@ -17899,7 +17896,7 @@
       <c r="BR91" s="10"/>
       <c r="BS91" s="10"/>
     </row>
-    <row r="92" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>71</v>
       </c>
@@ -18080,7 +18077,7 @@
       <c r="BR92" s="10"/>
       <c r="BS92" s="10"/>
     </row>
-    <row r="93" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>72</v>
       </c>
@@ -18261,7 +18258,7 @@
       <c r="BR93" s="10"/>
       <c r="BS93" s="10"/>
     </row>
-    <row r="94" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>70</v>
       </c>
@@ -18476,7 +18473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>71</v>
       </c>
@@ -18657,7 +18654,7 @@
       <c r="BR95" s="10"/>
       <c r="BS95" s="10"/>
     </row>
-    <row r="96" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>71</v>
       </c>
@@ -18838,7 +18835,7 @@
       <c r="BR96" s="10"/>
       <c r="BS96" s="10"/>
     </row>
-    <row r="97" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>71</v>
       </c>
@@ -19019,7 +19016,7 @@
       <c r="BR97" s="10"/>
       <c r="BS97" s="10"/>
     </row>
-    <row r="98" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>70</v>
       </c>
@@ -19200,7 +19197,7 @@
       <c r="BR98" s="10"/>
       <c r="BS98" s="10"/>
     </row>
-    <row r="99" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>71</v>
       </c>
@@ -19381,7 +19378,7 @@
       <c r="BR99" s="10"/>
       <c r="BS99" s="10"/>
     </row>
-    <row r="100" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>71</v>
       </c>
@@ -19596,7 +19593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>70</v>
       </c>
@@ -19777,7 +19774,7 @@
       <c r="BR101" s="10"/>
       <c r="BS101" s="10"/>
     </row>
-    <row r="102" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>71</v>
       </c>
@@ -19992,7 +19989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>70</v>
       </c>
@@ -20207,7 +20204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>71</v>
       </c>
@@ -20422,7 +20419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>70</v>
       </c>
@@ -20637,7 +20634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>71</v>
       </c>
@@ -20852,7 +20849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>72</v>
       </c>
@@ -21067,7 +21064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>72</v>
       </c>
@@ -21282,7 +21279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>72</v>
       </c>
@@ -21463,7 +21460,7 @@
       <c r="BR109" s="10"/>
       <c r="BS109" s="10"/>
     </row>
-    <row r="110" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>71</v>
       </c>
@@ -21678,7 +21675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>70</v>
       </c>
@@ -21893,7 +21890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>72</v>
       </c>
@@ -22108,7 +22105,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>72</v>
       </c>
@@ -22323,7 +22320,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>72</v>
       </c>
@@ -22538,7 +22535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>70</v>
       </c>
@@ -22753,7 +22750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>71</v>
       </c>
@@ -22968,7 +22965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>72</v>
       </c>
@@ -23183,7 +23180,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>70</v>
       </c>
@@ -23398,7 +23395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>72</v>
       </c>
@@ -23579,7 +23576,7 @@
       <c r="BR119" s="10"/>
       <c r="BS119" s="10"/>
     </row>
-    <row r="120" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>70</v>
       </c>
@@ -23794,7 +23791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>71</v>
       </c>
@@ -24009,7 +24006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>71</v>
       </c>
@@ -24224,7 +24221,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>72</v>
       </c>
@@ -24405,7 +24402,7 @@
       <c r="BR123" s="10"/>
       <c r="BS123" s="10"/>
     </row>
-    <row r="124" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>71</v>
       </c>
@@ -24586,7 +24583,7 @@
       <c r="BR124" s="10"/>
       <c r="BS124" s="10"/>
     </row>
-    <row r="125" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>70</v>
       </c>
@@ -24801,7 +24798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>72</v>
       </c>
@@ -24982,7 +24979,7 @@
       <c r="BR126" s="10"/>
       <c r="BS126" s="10"/>
     </row>
-    <row r="127" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>71</v>
       </c>
@@ -25163,7 +25160,7 @@
       <c r="BR127" s="10"/>
       <c r="BS127" s="10"/>
     </row>
-    <row r="128" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>72</v>
       </c>
@@ -25378,7 +25375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>70</v>
       </c>
@@ -25559,7 +25556,7 @@
       <c r="BR129" s="10"/>
       <c r="BS129" s="10"/>
     </row>
-    <row r="130" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>70</v>
       </c>
@@ -25774,7 +25771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>71</v>
       </c>
@@ -25989,7 +25986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>70</v>
       </c>
@@ -26170,7 +26167,7 @@
       <c r="BR132" s="10"/>
       <c r="BS132" s="10"/>
     </row>
-    <row r="133" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>70</v>
       </c>
@@ -26385,7 +26382,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>70</v>
       </c>
@@ -26600,7 +26597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>72</v>
       </c>
@@ -26781,7 +26778,7 @@
       <c r="BR135" s="10"/>
       <c r="BS135" s="10"/>
     </row>
-    <row r="136" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>71</v>
       </c>
@@ -26996,7 +26993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>71</v>
       </c>
@@ -27211,7 +27208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>70</v>
       </c>
@@ -27426,7 +27423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>71</v>
       </c>
@@ -27641,7 +27638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>71</v>
       </c>
@@ -27822,7 +27819,7 @@
       <c r="BR140" s="10"/>
       <c r="BS140" s="10"/>
     </row>
-    <row r="141" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>71</v>
       </c>
@@ -28037,7 +28034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>72</v>
       </c>
@@ -28252,7 +28249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>72</v>
       </c>
@@ -28467,7 +28464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>70</v>
       </c>
@@ -28648,7 +28645,7 @@
       <c r="BR144" s="10"/>
       <c r="BS144" s="10"/>
     </row>
-    <row r="145" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>72</v>
       </c>
@@ -28863,7 +28860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>71</v>
       </c>
@@ -29078,7 +29075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>72</v>
       </c>
@@ -29293,7 +29290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>71</v>
       </c>
@@ -29508,7 +29505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>70</v>
       </c>
@@ -29723,7 +29720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>70</v>
       </c>
@@ -29904,7 +29901,7 @@
       <c r="BR150" s="10"/>
       <c r="BS150" s="10"/>
     </row>
-    <row r="151" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>72</v>
       </c>
@@ -30085,7 +30082,7 @@
       <c r="BR151" s="10"/>
       <c r="BS151" s="10"/>
     </row>
-    <row r="152" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>70</v>
       </c>
@@ -30266,7 +30263,7 @@
       <c r="BR152" s="10"/>
       <c r="BS152" s="10"/>
     </row>
-    <row r="153" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>70</v>
       </c>
@@ -30481,7 +30478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>72</v>
       </c>
@@ -30696,7 +30693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>71</v>
       </c>
@@ -30911,7 +30908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>71</v>
       </c>
@@ -31126,7 +31123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>70</v>
       </c>
@@ -31341,7 +31338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>72</v>
       </c>
@@ -31522,7 +31519,7 @@
       <c r="BR158" s="10"/>
       <c r="BS158" s="10"/>
     </row>
-    <row r="159" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>72</v>
       </c>
@@ -31737,7 +31734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>70</v>
       </c>
@@ -31952,7 +31949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>72</v>
       </c>
@@ -32167,7 +32164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>71</v>
       </c>
@@ -32382,7 +32379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>70</v>
       </c>
@@ -32597,7 +32594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>70</v>
       </c>
@@ -32812,7 +32809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>70</v>
       </c>
@@ -33027,7 +33024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>71</v>
       </c>
@@ -33242,7 +33239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>71</v>
       </c>
@@ -33457,7 +33454,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>71</v>
       </c>
@@ -33672,7 +33669,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>72</v>
       </c>
@@ -33887,7 +33884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>70</v>
       </c>
@@ -34102,7 +34099,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>71</v>
       </c>
@@ -34317,7 +34314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>71</v>
       </c>
@@ -34532,7 +34529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>71</v>
       </c>
@@ -34747,7 +34744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>71</v>
       </c>
@@ -34962,7 +34959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>71</v>
       </c>
@@ -35177,7 +35174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>72</v>
       </c>
@@ -35392,7 +35389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>70</v>
       </c>
@@ -35607,7 +35604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>70</v>
       </c>
@@ -35822,7 +35819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:71" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>72</v>
       </c>

</xml_diff>